<commit_message>
Use angle-dependent shapes in SOT model curves
</commit_message>
<xml_diff>
--- a/SOT_results/SOT_0deg.xlsx
+++ b/SOT_results/SOT_0deg.xlsx
@@ -152,7 +152,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>0° 模型数据（52点）</a:t>
+              <a:t>0° 模型数据（角度相关形状，52点）</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -181,7 +181,7 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Sheet1'!$A$2:$A$53</f>
+              <f>'Sheet1'!$A$2:$A$27</f>
             </numRef>
           </xVal>
           <yVal>
@@ -625,7 +625,7 @@
         <v>-0.035</v>
       </c>
       <c r="B2" t="n">
-        <v>16.90153589494063</v>
+        <v>17.47943486872997</v>
       </c>
     </row>
     <row r="3">
@@ -633,7 +633,7 @@
         <v>-0.0322</v>
       </c>
       <c r="B3" t="n">
-        <v>16.88230956040268</v>
+        <v>17.10272421664234</v>
       </c>
     </row>
     <row r="4">
@@ -641,7 +641,7 @@
         <v>-0.0294</v>
       </c>
       <c r="B4" t="n">
-        <v>16.88094840397522</v>
+        <v>16.80418393457441</v>
       </c>
     </row>
     <row r="5">
@@ -649,7 +649,7 @@
         <v>-0.0266</v>
       </c>
       <c r="B5" t="n">
-        <v>16.88060811486835</v>
+        <v>16.83684697057579</v>
       </c>
     </row>
     <row r="6">
@@ -657,7 +657,7 @@
         <v>-0.0238</v>
       </c>
       <c r="B6" t="n">
-        <v>16.88111854852865</v>
+        <v>16.89469536107498</v>
       </c>
     </row>
     <row r="7">
@@ -665,7 +665,7 @@
         <v>-0.021</v>
       </c>
       <c r="B7" t="n">
-        <v>16.88026782576149</v>
+        <v>16.89952936182164</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +673,7 @@
         <v>-0.0182</v>
       </c>
       <c r="B8" t="n">
-        <v>16.87992753665462</v>
+        <v>16.87219303771848</v>
       </c>
     </row>
     <row r="9">
@@ -681,7 +681,7 @@
         <v>-0.0154</v>
       </c>
       <c r="B9" t="n">
-        <v>16.88196927129582</v>
+        <v>16.87124308618445</v>
       </c>
     </row>
     <row r="10">
@@ -689,7 +689,7 @@
         <v>-0.0126</v>
       </c>
       <c r="B10" t="n">
-        <v>16.88026782576149</v>
+        <v>16.87043280080362</v>
       </c>
     </row>
     <row r="11">
@@ -697,7 +697,7 @@
         <v>-0.0098</v>
       </c>
       <c r="B11" t="n">
-        <v>16.88435129504388</v>
+        <v>16.86388013044959</v>
       </c>
     </row>
     <row r="12">
@@ -705,7 +705,7 @@
         <v>-0.007</v>
       </c>
       <c r="B12" t="n">
-        <v>16.88281999406298</v>
+        <v>16.85969901354604</v>
       </c>
     </row>
     <row r="13">
@@ -713,7 +713,7 @@
         <v>-0.0042</v>
       </c>
       <c r="B13" t="n">
-        <v>16.88111854852865</v>
+        <v>16.86149527546073</v>
       </c>
     </row>
     <row r="14">
@@ -721,7 +721,7 @@
         <v>-0.0014</v>
       </c>
       <c r="B14" t="n">
-        <v>16.88213941584925</v>
+        <v>16.86003709431369</v>
       </c>
     </row>
     <row r="15">
@@ -729,7 +729,7 @@
         <v>0.0014</v>
       </c>
       <c r="B15" t="n">
-        <v>16.88179912674238</v>
+        <v>16.85898959816473</v>
       </c>
     </row>
     <row r="16">
@@ -737,7 +737,7 @@
         <v>0.0042</v>
       </c>
       <c r="B16" t="n">
-        <v>16.88401100593702</v>
+        <v>16.85777638701655</v>
       </c>
     </row>
     <row r="17">
@@ -745,7 +745,7 @@
         <v>0.007</v>
       </c>
       <c r="B17" t="n">
-        <v>16.88537216236448</v>
+        <v>17.04785370805233</v>
       </c>
     </row>
     <row r="18">
@@ -753,7 +753,7 @@
         <v>0.0098</v>
       </c>
       <c r="B18" t="n">
-        <v>16.88401100593702</v>
+        <v>17.37541074190787</v>
       </c>
     </row>
     <row r="19">
@@ -761,7 +761,7 @@
         <v>0.0126</v>
       </c>
       <c r="B19" t="n">
-        <v>16.88520201781105</v>
+        <v>17.57173479791449</v>
       </c>
     </row>
     <row r="20">
@@ -769,7 +769,7 @@
         <v>0.0154</v>
       </c>
       <c r="B20" t="n">
-        <v>16.88605274057822</v>
+        <v>17.58320127824558</v>
       </c>
     </row>
     <row r="21">
@@ -777,7 +777,7 @@
         <v>0.0182</v>
       </c>
       <c r="B21" t="n">
-        <v>16.88486172870418</v>
+        <v>17.57560166597336</v>
       </c>
     </row>
     <row r="22">
@@ -785,7 +785,7 @@
         <v>0.021</v>
       </c>
       <c r="B22" t="n">
-        <v>16.88622288513165</v>
+        <v>17.5380569653794</v>
       </c>
     </row>
     <row r="23">
@@ -793,7 +793,7 @@
         <v>0.0238</v>
       </c>
       <c r="B23" t="n">
-        <v>16.88707360789881</v>
+        <v>17.48530971485639</v>
       </c>
     </row>
     <row r="24">
@@ -801,7 +801,7 @@
         <v>0.0266</v>
       </c>
       <c r="B24" t="n">
-        <v>16.89047649896747</v>
+        <v>17.10180253087741</v>
       </c>
     </row>
     <row r="25">
@@ -809,7 +809,7 @@
         <v>0.0294</v>
       </c>
       <c r="B25" t="n">
-        <v>16.90561936422302</v>
+        <v>17.3916253172168</v>
       </c>
     </row>
     <row r="26">
@@ -817,7 +817,7 @@
         <v>0.0322</v>
       </c>
       <c r="B26" t="n">
-        <v>16.96925342720702</v>
+        <v>17.59302945243047</v>
       </c>
     </row>
     <row r="27">
@@ -825,7 +825,7 @@
         <v>0.035</v>
       </c>
       <c r="B27" t="n">
-        <v>17.04173500696954</v>
+        <v>17.40216013562916</v>
       </c>
     </row>
     <row r="28">
@@ -833,7 +833,7 @@
         <v>0.035</v>
       </c>
       <c r="B28" t="n">
-        <v>17.01400144475994</v>
+        <v>17.40497230253911</v>
       </c>
     </row>
     <row r="29">
@@ -841,7 +841,7 @@
         <v>0.0322</v>
       </c>
       <c r="B29" t="n">
-        <v>17.02744286448116</v>
+        <v>17.4892259094535</v>
       </c>
     </row>
     <row r="30">
@@ -849,7 +849,7 @@
         <v>0.0294</v>
       </c>
       <c r="B30" t="n">
-        <v>17.03135618921012</v>
+        <v>17.41097185058803</v>
       </c>
     </row>
     <row r="31">
@@ -857,7 +857,7 @@
         <v>0.0266</v>
       </c>
       <c r="B31" t="n">
-        <v>17.04037385054207</v>
+        <v>17.64260871989134</v>
       </c>
     </row>
     <row r="32">
@@ -865,7 +865,7 @@
         <v>0.0238</v>
       </c>
       <c r="B32" t="n">
-        <v>17.03969327232834</v>
+        <v>17.65801744366556</v>
       </c>
     </row>
     <row r="33">
@@ -873,7 +873,7 @@
         <v>0.021</v>
       </c>
       <c r="B33" t="n">
-        <v>17.04037385054207</v>
+        <v>17.54056596805999</v>
       </c>
     </row>
     <row r="34">
@@ -881,7 +881,7 @@
         <v>0.0182</v>
       </c>
       <c r="B34" t="n">
-        <v>17.04394688616417</v>
+        <v>17.1117071889081</v>
       </c>
     </row>
     <row r="35">
@@ -889,7 +889,7 @@
         <v>0.0154</v>
       </c>
       <c r="B35" t="n">
-        <v>17.0425857297367</v>
+        <v>17.04424400306918</v>
       </c>
     </row>
     <row r="36">
@@ -897,7 +897,7 @@
         <v>0.0126</v>
       </c>
       <c r="B36" t="n">
-        <v>17.04496775348477</v>
+        <v>17.04272984461471</v>
       </c>
     </row>
     <row r="37">
@@ -905,7 +905,7 @@
         <v>0.0098</v>
       </c>
       <c r="B37" t="n">
-        <v>17.0482005</v>
+        <v>17.03027627928823</v>
       </c>
     </row>
     <row r="38">
@@ -913,7 +913,7 @@
         <v>0.007</v>
       </c>
       <c r="B38" t="n">
-        <v>17.0446274643779</v>
+        <v>17.02803275314485</v>
       </c>
     </row>
     <row r="39">
@@ -921,7 +921,7 @@
         <v>0.0042</v>
       </c>
       <c r="B39" t="n">
-        <v>17.04700948812597</v>
+        <v>17.02596713507758</v>
       </c>
     </row>
     <row r="40">
@@ -929,7 +929,7 @@
         <v>0.0014</v>
       </c>
       <c r="B40" t="n">
-        <v>17.0482005</v>
+        <v>17.02817740737495</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
         <v>-0.0014</v>
       </c>
       <c r="B41" t="n">
-        <v>17.05568686035106</v>
+        <v>17.02613672969217</v>
       </c>
     </row>
     <row r="42">
@@ -945,7 +945,7 @@
         <v>-0.0042</v>
       </c>
       <c r="B42" t="n">
-        <v>17.0482005</v>
+        <v>17.02222275201813</v>
       </c>
     </row>
     <row r="43">
@@ -953,7 +953,7 @@
         <v>-0.007</v>
       </c>
       <c r="B43" t="n">
-        <v>17.0492213673206</v>
+        <v>17.02068864125606</v>
       </c>
     </row>
     <row r="44">
@@ -961,7 +961,7 @@
         <v>-0.0098</v>
       </c>
       <c r="B44" t="n">
-        <v>17.04956165642746</v>
+        <v>17.01449067859268</v>
       </c>
     </row>
     <row r="45">
@@ -969,7 +969,7 @@
         <v>-0.0126</v>
       </c>
       <c r="B45" t="n">
-        <v>17.0492213673206</v>
+        <v>17.07331340677963</v>
       </c>
     </row>
     <row r="46">
@@ -977,7 +977,7 @@
         <v>-0.0154</v>
       </c>
       <c r="B46" t="n">
-        <v>17.04956165642746</v>
+        <v>17.18785129124496</v>
       </c>
     </row>
     <row r="47">
@@ -985,7 +985,7 @@
         <v>-0.0182</v>
       </c>
       <c r="B47" t="n">
-        <v>17.0487109336603</v>
+        <v>17.27457399622474</v>
       </c>
     </row>
     <row r="48">
@@ -993,7 +993,7 @@
         <v>-0.021</v>
       </c>
       <c r="B48" t="n">
-        <v>17.04837064455343</v>
+        <v>17.32125685369913</v>
       </c>
     </row>
     <row r="49">
@@ -1001,7 +1001,7 @@
         <v>-0.0238</v>
       </c>
       <c r="B49" t="n">
-        <v>17.04939151187403</v>
+        <v>17.11974187233213</v>
       </c>
     </row>
     <row r="50">
@@ -1009,7 +1009,7 @@
         <v>-0.0266</v>
       </c>
       <c r="B50" t="n">
-        <v>17.04598862080537</v>
+        <v>17.10853976007673</v>
       </c>
     </row>
     <row r="51">
@@ -1017,7 +1017,7 @@
         <v>-0.0294</v>
       </c>
       <c r="B51" t="n">
-        <v>17.02897416546205</v>
+        <v>17.12700506652899</v>
       </c>
     </row>
     <row r="52">
@@ -1025,7 +1025,7 @@
         <v>-0.0322</v>
       </c>
       <c r="B52" t="n">
-        <v>16.93896769669592</v>
+        <v>17.36856543770906</v>
       </c>
     </row>
     <row r="53">
@@ -1033,7 +1033,7 @@
         <v>-0.035</v>
       </c>
       <c r="B53" t="n">
-        <v>16.8448777586474</v>
+        <v>17.44820618195268</v>
       </c>
     </row>
   </sheetData>
@@ -1074,11 +1074,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1144,84 +1144,60 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>电阻单位</t>
+          <t>翻转幅度A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>沿用原始文件数值；原始文件未注明纵轴单位</t>
+          <t>0.164785（保持前次角度模型）</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>翻转幅度A</t>
+          <t>曲线形状</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.164785（按前次分析的平台差模型）</t>
+          <t>角度相关形状模板：0°/45°/75°实测回线归一化后按角度混合</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>中心基线</t>
+          <t>形状插值</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>16.965808（由已测角度基线保形插值，仅用于保持绘图尺度）</t>
+          <t>0°→45°线性混合</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>曲线形状</t>
+          <t>纵轴单位</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>复用165°实测回线的两支路形状，按目标角度A缩放；未添加随机噪声</t>
+          <t>原始文件未注明，保留原始数值尺度</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>模型规律</t>
+          <t>实测区分</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0–90°单峰角度依赖；采用0°/45°/75°/90°实测幅度锚点的保形插值</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>实测区分</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>本文件不是该角度的实测记录；15°、30°、60°原始文件夹无实测数据，0°和45°文件也已按52点序列重新模型化</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>输入模板</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>165度.xlsx（用户上传）</t>
+          <t>本文件为模型生成数据；15°、30°、60°无原始OPJU，0°/45°为统一点数并按实测模板生成</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate clean standard SOT model curves
</commit_message>
<xml_diff>
--- a/SOT_results/SOT_0deg.xlsx
+++ b/SOT_results/SOT_0deg.xlsx
@@ -152,7 +152,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>0° 模型数据（角度相关形状，52点）</a:t>
+              <a:t>0° 标准双支路SOT模型（52点）</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -625,7 +625,7 @@
         <v>-0.035</v>
       </c>
       <c r="B2" t="n">
-        <v>17.47943486872997</v>
+        <v>16.8834155</v>
       </c>
     </row>
     <row r="3">
@@ -633,7 +633,7 @@
         <v>-0.0322</v>
       </c>
       <c r="B3" t="n">
-        <v>17.10272421664234</v>
+        <v>16.8834155</v>
       </c>
     </row>
     <row r="4">
@@ -641,7 +641,7 @@
         <v>-0.0294</v>
       </c>
       <c r="B4" t="n">
-        <v>16.80418393457441</v>
+        <v>16.8834155</v>
       </c>
     </row>
     <row r="5">
@@ -649,7 +649,7 @@
         <v>-0.0266</v>
       </c>
       <c r="B5" t="n">
-        <v>16.83684697057579</v>
+        <v>16.8834155</v>
       </c>
     </row>
     <row r="6">
@@ -657,7 +657,7 @@
         <v>-0.0238</v>
       </c>
       <c r="B6" t="n">
-        <v>16.89469536107498</v>
+        <v>16.88341550000001</v>
       </c>
     </row>
     <row r="7">
@@ -665,7 +665,7 @@
         <v>-0.021</v>
       </c>
       <c r="B7" t="n">
-        <v>16.89952936182164</v>
+        <v>16.88341550000003</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +673,7 @@
         <v>-0.0182</v>
       </c>
       <c r="B8" t="n">
-        <v>16.87219303771848</v>
+        <v>16.88341550000014</v>
       </c>
     </row>
     <row r="9">
@@ -681,7 +681,7 @@
         <v>-0.0154</v>
       </c>
       <c r="B9" t="n">
-        <v>16.87124308618445</v>
+        <v>16.88341550000075</v>
       </c>
     </row>
     <row r="10">
@@ -689,7 +689,7 @@
         <v>-0.0126</v>
       </c>
       <c r="B10" t="n">
-        <v>16.87043280080362</v>
+        <v>16.88341550000388</v>
       </c>
     </row>
     <row r="11">
@@ -697,7 +697,7 @@
         <v>-0.0098</v>
       </c>
       <c r="B11" t="n">
-        <v>16.86388013044959</v>
+        <v>16.88341550002017</v>
       </c>
     </row>
     <row r="12">
@@ -705,7 +705,7 @@
         <v>-0.007</v>
       </c>
       <c r="B12" t="n">
-        <v>16.85969901354604</v>
+        <v>16.88341550010473</v>
       </c>
     </row>
     <row r="13">
@@ -713,7 +713,7 @@
         <v>-0.0042</v>
       </c>
       <c r="B13" t="n">
-        <v>16.86149527546073</v>
+        <v>16.88341550054375</v>
       </c>
     </row>
     <row r="14">
@@ -721,7 +721,7 @@
         <v>-0.0014</v>
       </c>
       <c r="B14" t="n">
-        <v>16.86003709431369</v>
+        <v>16.883415502823</v>
       </c>
     </row>
     <row r="15">
@@ -729,7 +729,7 @@
         <v>0.0014</v>
       </c>
       <c r="B15" t="n">
-        <v>16.85898959816473</v>
+        <v>16.88341551465612</v>
       </c>
     </row>
     <row r="16">
@@ -737,7 +737,7 @@
         <v>0.0042</v>
       </c>
       <c r="B16" t="n">
-        <v>16.85777638701655</v>
+        <v>16.88341557608996</v>
       </c>
     </row>
     <row r="17">
@@ -745,7 +745,7 @@
         <v>0.007</v>
       </c>
       <c r="B17" t="n">
-        <v>17.04785370805233</v>
+        <v>16.88341589503457</v>
       </c>
     </row>
     <row r="18">
@@ -753,7 +753,7 @@
         <v>0.0098</v>
       </c>
       <c r="B18" t="n">
-        <v>17.37541074190787</v>
+        <v>16.88341755087551</v>
       </c>
     </row>
     <row r="19">
@@ -761,7 +761,7 @@
         <v>0.0126</v>
       </c>
       <c r="B19" t="n">
-        <v>17.57173479791449</v>
+        <v>16.88342614694968</v>
       </c>
     </row>
     <row r="20">
@@ -769,7 +769,7 @@
         <v>0.0154</v>
       </c>
       <c r="B20" t="n">
-        <v>17.58320127824558</v>
+        <v>16.88347076067125</v>
       </c>
     </row>
     <row r="21">
@@ -777,7 +777,7 @@
         <v>0.0182</v>
       </c>
       <c r="B21" t="n">
-        <v>17.57560166597336</v>
+        <v>16.88370199342717</v>
       </c>
     </row>
     <row r="22">
@@ -785,7 +785,7 @@
         <v>0.021</v>
       </c>
       <c r="B22" t="n">
-        <v>17.5380569653794</v>
+        <v>16.88489212332209</v>
       </c>
     </row>
     <row r="23">
@@ -793,7 +793,7 @@
         <v>0.0238</v>
       </c>
       <c r="B23" t="n">
-        <v>17.48530971485639</v>
+        <v>16.89080413996444</v>
       </c>
     </row>
     <row r="24">
@@ -801,7 +801,7 @@
         <v>0.0266</v>
       </c>
       <c r="B24" t="n">
-        <v>17.10180253087741</v>
+        <v>16.91570608723391</v>
       </c>
     </row>
     <row r="25">
@@ -809,7 +809,7 @@
         <v>0.0294</v>
       </c>
       <c r="B25" t="n">
-        <v>17.3916253172168</v>
+        <v>16.97545676069531</v>
       </c>
     </row>
     <row r="26">
@@ -817,7 +817,7 @@
         <v>0.0322</v>
       </c>
       <c r="B26" t="n">
-        <v>17.59302945243047</v>
+        <v>17.02642929636333</v>
       </c>
     </row>
     <row r="27">
@@ -825,7 +825,7 @@
         <v>0.035</v>
       </c>
       <c r="B27" t="n">
-        <v>17.40216013562916</v>
+        <v>17.04350629231351</v>
       </c>
     </row>
     <row r="28">
@@ -833,7 +833,7 @@
         <v>0.035</v>
       </c>
       <c r="B28" t="n">
-        <v>17.40497230253911</v>
+        <v>17.0482005</v>
       </c>
     </row>
     <row r="29">
@@ -841,7 +841,7 @@
         <v>0.0322</v>
       </c>
       <c r="B29" t="n">
-        <v>17.4892259094535</v>
+        <v>17.0482005</v>
       </c>
     </row>
     <row r="30">
@@ -849,7 +849,7 @@
         <v>0.0294</v>
       </c>
       <c r="B30" t="n">
-        <v>17.41097185058803</v>
+        <v>17.0482005</v>
       </c>
     </row>
     <row r="31">
@@ -857,7 +857,7 @@
         <v>0.0266</v>
       </c>
       <c r="B31" t="n">
-        <v>17.64260871989134</v>
+        <v>17.0482005</v>
       </c>
     </row>
     <row r="32">
@@ -865,7 +865,7 @@
         <v>0.0238</v>
       </c>
       <c r="B32" t="n">
-        <v>17.65801744366556</v>
+        <v>17.04820049999999</v>
       </c>
     </row>
     <row r="33">
@@ -873,7 +873,7 @@
         <v>0.021</v>
       </c>
       <c r="B33" t="n">
-        <v>17.54056596805999</v>
+        <v>17.04820049999997</v>
       </c>
     </row>
     <row r="34">
@@ -881,7 +881,7 @@
         <v>0.0182</v>
       </c>
       <c r="B34" t="n">
-        <v>17.1117071889081</v>
+        <v>17.04820049999985</v>
       </c>
     </row>
     <row r="35">
@@ -889,7 +889,7 @@
         <v>0.0154</v>
       </c>
       <c r="B35" t="n">
-        <v>17.04424400306918</v>
+        <v>17.04820049999925</v>
       </c>
     </row>
     <row r="36">
@@ -897,7 +897,7 @@
         <v>0.0126</v>
       </c>
       <c r="B36" t="n">
-        <v>17.04272984461471</v>
+        <v>17.04820049999611</v>
       </c>
     </row>
     <row r="37">
@@ -905,7 +905,7 @@
         <v>0.0098</v>
       </c>
       <c r="B37" t="n">
-        <v>17.03027627928823</v>
+        <v>17.04820049997982</v>
       </c>
     </row>
     <row r="38">
@@ -913,7 +913,7 @@
         <v>0.007</v>
       </c>
       <c r="B38" t="n">
-        <v>17.02803275314485</v>
+        <v>17.04820049989526</v>
       </c>
     </row>
     <row r="39">
@@ -921,7 +921,7 @@
         <v>0.0042</v>
       </c>
       <c r="B39" t="n">
-        <v>17.02596713507758</v>
+        <v>17.04820049945624</v>
       </c>
     </row>
     <row r="40">
@@ -929,7 +929,7 @@
         <v>0.0014</v>
       </c>
       <c r="B40" t="n">
-        <v>17.02817740737495</v>
+        <v>17.048200497177</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
         <v>-0.0014</v>
       </c>
       <c r="B41" t="n">
-        <v>17.02613672969217</v>
+        <v>17.04820048534388</v>
       </c>
     </row>
     <row r="42">
@@ -945,7 +945,7 @@
         <v>-0.0042</v>
       </c>
       <c r="B42" t="n">
-        <v>17.02222275201813</v>
+        <v>17.04820042391003</v>
       </c>
     </row>
     <row r="43">
@@ -953,7 +953,7 @@
         <v>-0.007</v>
       </c>
       <c r="B43" t="n">
-        <v>17.02068864125606</v>
+        <v>17.04820010496543</v>
       </c>
     </row>
     <row r="44">
@@ -961,7 +961,7 @@
         <v>-0.0098</v>
       </c>
       <c r="B44" t="n">
-        <v>17.01449067859268</v>
+        <v>17.04819844912449</v>
       </c>
     </row>
     <row r="45">
@@ -969,7 +969,7 @@
         <v>-0.0126</v>
       </c>
       <c r="B45" t="n">
-        <v>17.07331340677963</v>
+        <v>17.04818985305032</v>
       </c>
     </row>
     <row r="46">
@@ -977,7 +977,7 @@
         <v>-0.0154</v>
       </c>
       <c r="B46" t="n">
-        <v>17.18785129124496</v>
+        <v>17.04814523932875</v>
       </c>
     </row>
     <row r="47">
@@ -985,7 +985,7 @@
         <v>-0.0182</v>
       </c>
       <c r="B47" t="n">
-        <v>17.27457399622474</v>
+        <v>17.04791400657282</v>
       </c>
     </row>
     <row r="48">
@@ -993,7 +993,7 @@
         <v>-0.021</v>
       </c>
       <c r="B48" t="n">
-        <v>17.32125685369913</v>
+        <v>17.04672387667791</v>
       </c>
     </row>
     <row r="49">
@@ -1001,7 +1001,7 @@
         <v>-0.0238</v>
       </c>
       <c r="B49" t="n">
-        <v>17.11974187233213</v>
+        <v>17.04081186003555</v>
       </c>
     </row>
     <row r="50">
@@ -1009,7 +1009,7 @@
         <v>-0.0266</v>
       </c>
       <c r="B50" t="n">
-        <v>17.10853976007673</v>
+        <v>17.01590991276608</v>
       </c>
     </row>
     <row r="51">
@@ -1017,7 +1017,7 @@
         <v>-0.0294</v>
       </c>
       <c r="B51" t="n">
-        <v>17.12700506652899</v>
+        <v>16.95615923930469</v>
       </c>
     </row>
     <row r="52">
@@ -1025,7 +1025,7 @@
         <v>-0.0322</v>
       </c>
       <c r="B52" t="n">
-        <v>17.36856543770906</v>
+        <v>16.90518670363667</v>
       </c>
     </row>
     <row r="53">
@@ -1033,7 +1033,7 @@
         <v>-0.035</v>
       </c>
       <c r="B53" t="n">
-        <v>17.44820618195268</v>
+        <v>16.88810970768649</v>
       </c>
     </row>
   </sheetData>
@@ -1074,11 +1074,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>模型生成（非实测）</t>
+          <t>标准双支路模型生成（非实测）</t>
         </is>
       </c>
     </row>
@@ -1149,55 +1149,67 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.164785（保持前次角度模型）</t>
+          <t>0.164785</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>曲线形状</t>
+          <t>开关阈值Ic</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>角度相关形状模板：0°/45°/75°实测回线归一化后按角度混合</t>
+          <t>±0.02900000 A（平滑角度模型）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>形状插值</t>
+          <t>开关宽度</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0°→45°线性混合</t>
+          <t>0.00170000 A（窄开关区）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>纵轴单位</t>
+          <t>曲线结构</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>原始文件未注明，保留原始数值尺度</t>
+          <t>支路1在+Ic由低平台翻到高平台；支路2在−Ic由高平台翻到低平台</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>噪声处理</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>未添加随机噪声；未使用原始回线端点噪声</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>实测区分</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>本文件为模型生成数据；15°、30°、60°无原始OPJU，0°/45°为统一点数并按实测模板生成</t>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>本文件是模型预测/标准化数据，不是该角度的原始实测记录</t>
         </is>
       </c>
     </row>

</xml_diff>